<commit_message>
week 2 add on
</commit_message>
<xml_diff>
--- a/data/leagues/Campers and Skiers and Prahlad 2026.xlsx
+++ b/data/leagues/Campers and Skiers and Prahlad 2026.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="98">
   <si>
     <t>Michael the International Baker</t>
   </si>
@@ -55,10 +55,13 @@
     <t>The Turbanator</t>
   </si>
   <si>
-    <t>0-1-0</t>
-  </si>
-  <si>
-    <t>1-0-0</t>
+    <t>0-2-0</t>
+  </si>
+  <si>
+    <t>1-1-0</t>
+  </si>
+  <si>
+    <t>2-0-0</t>
   </si>
   <si>
     <t>Teams</t>
@@ -118,6 +121,9 @@
     <t>Week_2</t>
   </si>
   <si>
+    <t>Week_3</t>
+  </si>
+  <si>
     <t>Owner</t>
   </si>
   <si>
@@ -139,36 +145,36 @@
     <t>Games_Remaining</t>
   </si>
   <si>
+    <t>Marvin Ta</t>
+  </si>
+  <si>
     <t>Anthony Rizzo</t>
   </si>
   <si>
+    <t>Maulin Patel</t>
+  </si>
+  <si>
+    <t>Chris Carbone</t>
+  </si>
+  <si>
     <t>Alyssa Ianovale</t>
   </si>
   <si>
-    <t>Marvin Ta</t>
+    <t>Victor Rojas</t>
+  </si>
+  <si>
+    <t>Robbie Wilston</t>
+  </si>
+  <si>
+    <t>Prahlad Singh</t>
   </si>
   <si>
     <t>Kermelos Woldeyes</t>
   </si>
   <si>
-    <t>Robbie Wilston</t>
-  </si>
-  <si>
-    <t>Maulin Patel</t>
-  </si>
-  <si>
-    <t>Chris Carbone</t>
-  </si>
-  <si>
-    <t>Victor Rojas</t>
-  </si>
-  <si>
     <t>Bridget Cashel</t>
   </si>
   <si>
-    <t>Prahlad Singh</t>
-  </si>
-  <si>
     <t>Current_Record</t>
   </si>
   <si>
@@ -193,51 +199,51 @@
     <t>Most_Likely_Record</t>
   </si>
   <si>
-    <t>1-0</t>
-  </si>
-  <si>
-    <t>0-1</t>
-  </si>
-  <si>
-    <t>10.6-3.3-0.1</t>
-  </si>
-  <si>
-    <t>9.4-4.6-0.1</t>
-  </si>
-  <si>
-    <t>9.3-4.6-0.1</t>
-  </si>
-  <si>
-    <t>9.2-4.7-0.1</t>
-  </si>
-  <si>
-    <t>7.0-6.9-0.1</t>
-  </si>
-  <si>
-    <t>6.6-7.3-0.1</t>
+    <t>1-1</t>
+  </si>
+  <si>
+    <t>2-0</t>
+  </si>
+  <si>
+    <t>0-2</t>
+  </si>
+  <si>
+    <t>9.7-4.2-0.1</t>
+  </si>
+  <si>
+    <t>8.1-5.8-0.1</t>
+  </si>
+  <si>
+    <t>8.2-5.7-0.1</t>
+  </si>
+  <si>
+    <t>7.7-6.2-0.1</t>
+  </si>
+  <si>
+    <t>7.2-6.7-0.1</t>
   </si>
   <si>
     <t>5.8-8.1-0.1</t>
   </si>
   <si>
-    <t>5.6-8.3-0.1</t>
+    <t>5.6-8.4-0.1</t>
+  </si>
+  <si>
+    <t>4.9-9.0-0.1</t>
   </si>
   <si>
     <t>4.3-9.6-0.1</t>
   </si>
   <si>
-    <t>1.8-12.1-0.1</t>
-  </si>
-  <si>
-    <t>11-3</t>
-  </si>
-  <si>
     <t>10-4</t>
   </si>
   <si>
     <t>9-5</t>
   </si>
   <si>
+    <t>8-6</t>
+  </si>
+  <si>
     <t>7-7</t>
   </si>
   <si>
@@ -250,9 +256,6 @@
     <t>4-10</t>
   </si>
   <si>
-    <t>1-13</t>
-  </si>
-  <si>
     <t>Owners</t>
   </si>
   <si>
@@ -262,7 +265,37 @@
     <t>Change From Last Week</t>
   </si>
   <si>
+    <t>↑10</t>
+  </si>
+  <si>
+    <t>↑8</t>
+  </si>
+  <si>
+    <t>↓1</t>
+  </si>
+  <si>
+    <t>↓2</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>↓3</t>
+  </si>
+  <si>
+    <t>↑2</t>
+  </si>
+  <si>
+    <t>↓5</t>
+  </si>
+  <si>
+    <t>↓7</t>
+  </si>
+  <si>
     <t>Week 1</t>
+  </si>
+  <si>
+    <t>Week 2</t>
   </si>
   <si>
     <t>Week</t>
@@ -684,7 +717,7 @@
         <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
         <v>10</v>
@@ -719,13 +752,13 @@
         <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F3" t="s">
         <v>10</v>
@@ -734,13 +767,13 @@
         <v>10</v>
       </c>
       <c r="H3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I3" t="s">
         <v>11</v>
       </c>
       <c r="J3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K3" t="s">
         <v>11</v>
@@ -754,13 +787,13 @@
         <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F4" t="s">
         <v>10</v>
@@ -769,13 +802,13 @@
         <v>10</v>
       </c>
       <c r="H4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K4" t="s">
         <v>11</v>
@@ -786,16 +819,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F5" t="s">
         <v>10</v>
@@ -804,16 +837,16 @@
         <v>10</v>
       </c>
       <c r="H5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -821,16 +854,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F6" t="s">
         <v>10</v>
@@ -839,16 +872,16 @@
         <v>10</v>
       </c>
       <c r="H6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -856,34 +889,34 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -894,13 +927,13 @@
         <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F8" t="s">
         <v>10</v>
@@ -909,16 +942,16 @@
         <v>10</v>
       </c>
       <c r="H8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -929,13 +962,13 @@
         <v>11</v>
       </c>
       <c r="C9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
       </c>
       <c r="E9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F9" t="s">
         <v>11</v>
@@ -999,13 +1032,13 @@
         <v>11</v>
       </c>
       <c r="C11" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D11" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E11" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F11" t="s">
         <v>10</v>
@@ -1033,30 +1066,56 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="B1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="2:8">
+    <row r="1" spans="1:8">
       <c r="B1" s="1" t="s">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>86</v>
+        <v>97</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" s="1">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2">
+        <v>-2</v>
+      </c>
+      <c r="F2">
+        <v>5</v>
+      </c>
+      <c r="G2">
+        <v>7</v>
+      </c>
+      <c r="H2" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -1071,13 +1130,13 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="B1" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -1088,7 +1147,7 @@
         <v>4</v>
       </c>
       <c r="C2">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="D2" t="s">
         <v>10</v>
@@ -1102,10 +1161,10 @@
         <v>5</v>
       </c>
       <c r="C3">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="D3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -1113,13 +1172,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C4">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="D4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -1127,10 +1186,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="C5">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="D5" t="s">
         <v>10</v>
@@ -1141,10 +1200,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C6">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="D6" t="s">
         <v>11</v>
@@ -1155,10 +1214,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C7">
-        <v>0.5</v>
+        <v>1.1</v>
       </c>
       <c r="D7" t="s">
         <v>11</v>
@@ -1169,13 +1228,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C8">
-        <v>0.7</v>
+        <v>1.2</v>
       </c>
       <c r="D8" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -1186,7 +1245,7 @@
         <v>8</v>
       </c>
       <c r="C9">
-        <v>0.7</v>
+        <v>1.3</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
@@ -1197,10 +1256,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C10">
-        <v>0.8</v>
+        <v>1.4</v>
       </c>
       <c r="D10" t="s">
         <v>11</v>
@@ -1211,13 +1270,13 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C11">
-        <v>0.9</v>
+        <v>1.7</v>
       </c>
       <c r="D11" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -1232,16 +1291,16 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="B1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -1249,13 +1308,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E2" t="s">
         <v>11</v>
@@ -1266,16 +1325,16 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C3">
-        <v>0.9</v>
+        <v>1.4</v>
       </c>
       <c r="D3">
-        <v>-0.09999999999999998</v>
+        <v>-0.6000000000000001</v>
       </c>
       <c r="E3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -1283,16 +1342,16 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C4">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="D4">
-        <v>-0.2</v>
+        <v>-0.8</v>
       </c>
       <c r="E4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -1300,13 +1359,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C5">
-        <v>0.7</v>
+        <v>1.2</v>
       </c>
       <c r="D5">
-        <v>-0.3</v>
+        <v>0.2</v>
       </c>
       <c r="E5" t="s">
         <v>11</v>
@@ -1317,16 +1376,16 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C6">
-        <v>0.5</v>
+        <v>1.2</v>
       </c>
       <c r="D6">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="E6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -1334,13 +1393,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C7">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="D7">
-        <v>-0.6</v>
+        <v>0.2</v>
       </c>
       <c r="E7" t="s">
         <v>11</v>
@@ -1351,16 +1410,16 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C8">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="D8">
-        <v>0.4</v>
+        <v>-0.2</v>
       </c>
       <c r="E8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -1368,13 +1427,13 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C9">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="D9">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="E9" t="s">
         <v>10</v>
@@ -1385,16 +1444,16 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C10">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="D10">
-        <v>0.1</v>
+        <v>-0.6</v>
       </c>
       <c r="E10" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -1402,13 +1461,13 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C11">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="D11">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="E11" t="s">
         <v>10</v>
@@ -1426,116 +1485,116 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2">
+        <v>53.3</v>
+      </c>
+      <c r="C2">
+        <v>20.5</v>
+      </c>
+      <c r="D2">
+        <v>12.4</v>
+      </c>
+      <c r="E2">
         <v>7</v>
       </c>
-      <c r="B2">
-        <v>54.5</v>
-      </c>
-      <c r="C2">
-        <v>22.2</v>
-      </c>
-      <c r="D2">
-        <v>12.3</v>
-      </c>
-      <c r="E2">
-        <v>6.8</v>
-      </c>
       <c r="F2">
-        <v>2.9</v>
+        <v>3.1</v>
       </c>
       <c r="G2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H2">
-        <v>0.1</v>
+        <v>1.2</v>
       </c>
       <c r="I2">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="J2">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K2">
         <v>0</v>
       </c>
       <c r="L2">
-        <v>99.7</v>
+        <v>98.3</v>
       </c>
     </row>
     <row r="3" spans="1:12">
       <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>10.2</v>
+      </c>
+      <c r="C3">
+        <v>19.3</v>
+      </c>
+      <c r="D3">
+        <v>18.5</v>
+      </c>
+      <c r="E3">
+        <v>15.5</v>
+      </c>
+      <c r="F3">
+        <v>15</v>
+      </c>
+      <c r="G3">
         <v>9</v>
       </c>
-      <c r="B3">
-        <v>15.5</v>
-      </c>
-      <c r="C3">
-        <v>24.3</v>
-      </c>
-      <c r="D3">
-        <v>23.2</v>
-      </c>
-      <c r="E3">
-        <v>20.3</v>
-      </c>
-      <c r="F3">
-        <v>9.9</v>
-      </c>
-      <c r="G3">
-        <v>4.2</v>
-      </c>
       <c r="H3">
-        <v>1.8</v>
+        <v>6.9</v>
       </c>
       <c r="I3">
-        <v>0.6</v>
+        <v>3.3</v>
       </c>
       <c r="J3">
-        <v>0.2</v>
+        <v>1.5</v>
       </c>
       <c r="K3">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="L3">
-        <v>97.40000000000001</v>
+        <v>87.5</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -1543,37 +1602,37 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>15</v>
+        <v>11.2</v>
       </c>
       <c r="C4">
-        <v>23.9</v>
+        <v>17.2</v>
       </c>
       <c r="D4">
-        <v>24</v>
+        <v>14.8</v>
       </c>
       <c r="E4">
-        <v>21.1</v>
+        <v>18.7</v>
       </c>
       <c r="F4">
-        <v>9.1</v>
+        <v>15.2</v>
       </c>
       <c r="G4">
-        <v>3.8</v>
+        <v>10.2</v>
       </c>
       <c r="H4">
-        <v>2.1</v>
+        <v>6.1</v>
       </c>
       <c r="I4">
+        <v>4.1</v>
+      </c>
+      <c r="J4">
+        <v>1.7</v>
+      </c>
+      <c r="K4">
         <v>0.8</v>
       </c>
-      <c r="J4">
-        <v>0.2</v>
-      </c>
-      <c r="K4">
-        <v>0</v>
-      </c>
       <c r="L4">
-        <v>96.90000000000001</v>
+        <v>87.3</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -1581,265 +1640,265 @@
         <v>1</v>
       </c>
       <c r="B5">
-        <v>14.3</v>
+        <v>10.2</v>
       </c>
       <c r="C5">
-        <v>22.3</v>
+        <v>15</v>
       </c>
       <c r="D5">
-        <v>23.9</v>
+        <v>16.3</v>
       </c>
       <c r="E5">
-        <v>18.4</v>
+        <v>17.2</v>
       </c>
       <c r="F5">
-        <v>11.7</v>
+        <v>14.4</v>
       </c>
       <c r="G5">
-        <v>5.3</v>
+        <v>13.1</v>
       </c>
       <c r="H5">
-        <v>2.9</v>
+        <v>6.3</v>
       </c>
       <c r="I5">
-        <v>1</v>
+        <v>4.7</v>
       </c>
       <c r="J5">
-        <v>0.2</v>
+        <v>2.4</v>
       </c>
       <c r="K5">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="L5">
-        <v>95.90000000000001</v>
+        <v>86.2</v>
       </c>
     </row>
     <row r="6" spans="1:12">
       <c r="A6" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B6">
-        <v>0.3</v>
+        <v>8.9</v>
       </c>
       <c r="C6">
-        <v>3.1</v>
+        <v>12.4</v>
       </c>
       <c r="D6">
-        <v>7.2</v>
+        <v>17</v>
       </c>
       <c r="E6">
-        <v>14.2</v>
+        <v>16.3</v>
       </c>
       <c r="F6">
-        <v>23.4</v>
+        <v>13.9</v>
       </c>
       <c r="G6">
-        <v>22.8</v>
+        <v>10.5</v>
       </c>
       <c r="H6">
-        <v>16.4</v>
+        <v>10.3</v>
       </c>
       <c r="I6">
-        <v>8.199999999999999</v>
+        <v>5.8</v>
       </c>
       <c r="J6">
-        <v>4.1</v>
+        <v>3.6</v>
       </c>
       <c r="K6">
-        <v>0.3</v>
+        <v>1.3</v>
       </c>
       <c r="L6">
-        <v>71</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:12">
       <c r="A7" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B7">
-        <v>0.1</v>
+        <v>4.6</v>
       </c>
       <c r="C7">
-        <v>2.1</v>
+        <v>11</v>
       </c>
       <c r="D7">
-        <v>5.3</v>
+        <v>11.4</v>
       </c>
       <c r="E7">
-        <v>9</v>
+        <v>12.1</v>
       </c>
       <c r="F7">
-        <v>18.3</v>
+        <v>15.5</v>
       </c>
       <c r="G7">
-        <v>22.5</v>
+        <v>14.8</v>
       </c>
       <c r="H7">
-        <v>20.1</v>
+        <v>12.4</v>
       </c>
       <c r="I7">
-        <v>15</v>
+        <v>9.6</v>
       </c>
       <c r="J7">
-        <v>7.1</v>
+        <v>5.9</v>
       </c>
       <c r="K7">
-        <v>0.5</v>
+        <v>2.7</v>
       </c>
       <c r="L7">
-        <v>57.3</v>
+        <v>69.40000000000001</v>
       </c>
     </row>
     <row r="8" spans="1:12">
       <c r="A8" s="1" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B8">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="C8">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="D8">
-        <v>3</v>
+        <v>3.4</v>
       </c>
       <c r="E8">
-        <v>5.1</v>
+        <v>4.9</v>
       </c>
       <c r="F8">
-        <v>12.2</v>
+        <v>8</v>
       </c>
       <c r="G8">
-        <v>18.3</v>
+        <v>16.1</v>
       </c>
       <c r="H8">
-        <v>20.9</v>
+        <v>21.7</v>
       </c>
       <c r="I8">
-        <v>22.7</v>
+        <v>21.5</v>
       </c>
       <c r="J8">
-        <v>14.5</v>
+        <v>13.9</v>
       </c>
       <c r="K8">
-        <v>2.1</v>
+        <v>8.9</v>
       </c>
       <c r="L8">
-        <v>39.8</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:12">
       <c r="A9" s="1" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B9">
-        <v>0.2</v>
+        <v>1.2</v>
       </c>
       <c r="C9">
-        <v>0.9</v>
+        <v>2.3</v>
       </c>
       <c r="D9">
-        <v>1.1</v>
+        <v>4</v>
       </c>
       <c r="E9">
-        <v>4.5</v>
+        <v>5.3</v>
       </c>
       <c r="F9">
-        <v>8.9</v>
+        <v>8.5</v>
       </c>
       <c r="G9">
-        <v>16</v>
+        <v>11.9</v>
       </c>
       <c r="H9">
-        <v>23.7</v>
+        <v>15.4</v>
       </c>
       <c r="I9">
-        <v>27.1</v>
+        <v>16.9</v>
       </c>
       <c r="J9">
-        <v>15.2</v>
+        <v>19</v>
       </c>
       <c r="K9">
-        <v>2.4</v>
+        <v>15.5</v>
       </c>
       <c r="L9">
-        <v>31.6</v>
+        <v>33.2</v>
       </c>
     </row>
     <row r="10" spans="1:12">
       <c r="A10" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B10">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="C10">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="D10">
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="E10">
-        <v>0.6</v>
+        <v>1.5</v>
       </c>
       <c r="F10">
-        <v>3.6</v>
+        <v>4</v>
       </c>
       <c r="G10">
-        <v>5.9</v>
+        <v>6.6</v>
       </c>
       <c r="H10">
-        <v>11.6</v>
+        <v>12</v>
       </c>
       <c r="I10">
-        <v>22.6</v>
+        <v>18.2</v>
       </c>
       <c r="J10">
-        <v>46.5</v>
+        <v>24.9</v>
       </c>
       <c r="K10">
-        <v>9.1</v>
+        <v>30.7</v>
       </c>
       <c r="L10">
-        <v>10.2</v>
+        <v>14.2</v>
       </c>
     </row>
     <row r="11" spans="1:12">
       <c r="A11" s="1" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B11">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="C11">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D11">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="E11">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="F11">
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="G11">
-        <v>0.2</v>
+        <v>5.8</v>
       </c>
       <c r="H11">
-        <v>0.4</v>
+        <v>7.7</v>
       </c>
       <c r="I11">
-        <v>1.9</v>
+        <v>15.4</v>
       </c>
       <c r="J11">
-        <v>11.9</v>
+        <v>27.1</v>
       </c>
       <c r="K11">
-        <v>85.59999999999999</v>
+        <v>38.9</v>
       </c>
       <c r="L11">
-        <v>0.2</v>
+        <v>10.9</v>
       </c>
     </row>
   </sheetData>
@@ -1849,125 +1908,158 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:4">
       <c r="B1" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
+        <v>31</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B2">
-        <v>99.90000000000001</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="C2">
-        <v>99.90000000000001</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
+        <v>98.5</v>
+      </c>
+      <c r="D2">
+        <v>98.59999999999999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>37.9</v>
+      </c>
+      <c r="C3">
+        <v>90.2</v>
+      </c>
+      <c r="D3">
+        <v>88.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>97.39999999999999</v>
-      </c>
-      <c r="C3">
-        <v>97.59999999999999</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" s="1" t="s">
-        <v>9</v>
-      </c>
       <c r="B4">
-        <v>97.7</v>
+        <v>97.2</v>
       </c>
       <c r="C4">
-        <v>97.3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
+        <v>87.59999999999999</v>
+      </c>
+      <c r="D4">
+        <v>86.2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
       <c r="A5" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B5">
-        <v>98.8</v>
+        <v>97.39999999999999</v>
       </c>
       <c r="C5">
-        <v>96.3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
+        <v>88.5</v>
+      </c>
+      <c r="D5">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
       <c r="A6" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B6">
-        <v>69.5</v>
+        <v>99.8</v>
       </c>
       <c r="C6">
-        <v>73.40000000000001</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
+        <v>80.7</v>
+      </c>
+      <c r="D6">
+        <v>79.90000000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
       <c r="A7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7">
+        <v>97.09999999999999</v>
+      </c>
+      <c r="C7">
+        <v>73.7</v>
+      </c>
+      <c r="D7">
+        <v>71.89999999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8">
+        <v>8.799999999999999</v>
+      </c>
+      <c r="C8">
+        <v>31.2</v>
+      </c>
+      <c r="D8">
+        <v>34.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9">
+        <v>0.1</v>
+      </c>
+      <c r="C9">
+        <v>27.1</v>
+      </c>
+      <c r="D9">
+        <v>30.7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B7">
-        <v>56.39999999999999</v>
-      </c>
-      <c r="C7">
-        <v>54.40000000000001</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8">
-        <v>38.1</v>
-      </c>
-      <c r="C8">
-        <v>38.2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" s="1" t="s">
+      <c r="B10">
+        <v>57.8</v>
+      </c>
+      <c r="C10">
+        <v>14.7</v>
+      </c>
+      <c r="D10">
+        <v>14.9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B9">
-        <v>33.6</v>
-      </c>
-      <c r="C9">
-        <v>34.7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B10">
-        <v>8.6</v>
-      </c>
-      <c r="C10">
-        <v>8.200000000000001</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3">
-      <c r="A11" s="1" t="s">
-        <v>4</v>
-      </c>
       <c r="B11">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="C11">
-        <v>0</v>
+        <v>7.8</v>
+      </c>
+      <c r="D11">
+        <v>8.799999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -1982,28 +2074,28 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="B1" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -2011,28 +2103,28 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D2">
-        <v>117.86</v>
+        <v>102.98</v>
       </c>
       <c r="E2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F2">
-        <v>125.63</v>
+        <v>124.15</v>
       </c>
       <c r="G2">
-        <v>0.538</v>
+        <v>0.5</v>
       </c>
       <c r="H2">
-        <v>0.8</v>
+        <v>2.3</v>
       </c>
       <c r="I2">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -2040,28 +2132,28 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="C3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D3">
-        <v>107</v>
+        <v>107.22</v>
       </c>
       <c r="E3" t="s">
         <v>10</v>
       </c>
       <c r="F3">
-        <v>126.97</v>
+        <v>122.38</v>
       </c>
       <c r="G3">
-        <v>0.538</v>
+        <v>0.542</v>
       </c>
       <c r="H3">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="I3">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -2069,28 +2161,28 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D4">
-        <v>118.96</v>
+        <v>122.45</v>
       </c>
       <c r="E4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F4">
-        <v>126.61</v>
+        <v>121.46</v>
       </c>
       <c r="G4">
-        <v>0.462</v>
+        <v>0.417</v>
       </c>
       <c r="H4">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="I4">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -2098,28 +2190,28 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D5">
-        <v>84.09999999999999</v>
+        <v>123.55</v>
       </c>
       <c r="E5" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F5">
-        <v>130.06</v>
+        <v>121.15</v>
       </c>
       <c r="G5">
-        <v>0.538</v>
+        <v>0.375</v>
       </c>
       <c r="H5">
-        <v>0.2</v>
+        <v>0.9</v>
       </c>
       <c r="I5">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -2127,28 +2219,28 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D6">
-        <v>155.66</v>
+        <v>113.89</v>
       </c>
       <c r="E6" t="s">
         <v>11</v>
       </c>
       <c r="F6">
-        <v>125.68</v>
+        <v>122.78</v>
       </c>
       <c r="G6">
-        <v>0.538</v>
+        <v>0.5</v>
       </c>
       <c r="H6">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="I6">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -2156,28 +2248,28 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D7">
-        <v>139.16</v>
+        <v>127.74</v>
       </c>
       <c r="E7" t="s">
         <v>11</v>
       </c>
       <c r="F7">
-        <v>122.35</v>
+        <v>120.05</v>
       </c>
       <c r="G7">
-        <v>0.462</v>
+        <v>0.542</v>
       </c>
       <c r="H7">
-        <v>-0.2</v>
+        <v>-0.3</v>
       </c>
       <c r="I7">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -2185,28 +2277,28 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D8">
-        <v>140.4</v>
+        <v>128.97</v>
       </c>
       <c r="E8" t="s">
         <v>11</v>
       </c>
       <c r="F8">
-        <v>122.67</v>
+        <v>119.39</v>
       </c>
       <c r="G8">
-        <v>0.385</v>
+        <v>0.5</v>
       </c>
       <c r="H8">
-        <v>-0.5</v>
+        <v>-0.6</v>
       </c>
       <c r="I8">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -2214,28 +2306,28 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D9">
-        <v>120.02</v>
+        <v>122.33</v>
       </c>
       <c r="E9" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F9">
-        <v>125.86</v>
+        <v>120.58</v>
       </c>
       <c r="G9">
-        <v>0.538</v>
+        <v>0.5</v>
       </c>
       <c r="H9">
-        <v>-0.5</v>
+        <v>-1.4</v>
       </c>
       <c r="I9">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -2243,28 +2335,28 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C10" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D10">
-        <v>126.56</v>
+        <v>113.63</v>
       </c>
       <c r="E10" t="s">
         <v>10</v>
       </c>
       <c r="F10">
-        <v>121.14</v>
+        <v>120.77</v>
       </c>
       <c r="G10">
-        <v>0.538</v>
+        <v>0.583</v>
       </c>
       <c r="H10">
-        <v>-0.7</v>
+        <v>-1.6</v>
       </c>
       <c r="I10">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -2272,28 +2364,28 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C11" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D11">
-        <v>141.2</v>
+        <v>146.89</v>
       </c>
       <c r="E11" t="s">
         <v>11</v>
       </c>
       <c r="F11">
-        <v>123.95</v>
+        <v>116.93</v>
       </c>
       <c r="G11">
-        <v>0.462</v>
+        <v>0.542</v>
       </c>
       <c r="H11">
-        <v>-0.9</v>
+        <v>-2.1</v>
       </c>
       <c r="I11">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -2308,89 +2400,89 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="D2">
-        <v>155.66</v>
+        <v>146.89</v>
       </c>
       <c r="E2">
-        <v>155.66</v>
+        <v>293.78</v>
       </c>
       <c r="F2">
-        <v>99.7</v>
+        <v>98.3</v>
       </c>
       <c r="G2">
         <v>0</v>
       </c>
       <c r="H2" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" s="1" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="D3">
-        <v>141.2</v>
+        <v>127.74</v>
       </c>
       <c r="E3">
-        <v>141.2</v>
+        <v>255.48</v>
       </c>
       <c r="F3">
-        <v>97.39999999999999</v>
+        <v>87.5</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="H3" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="I3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -2398,28 +2490,28 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C4">
         <v>1</v>
       </c>
       <c r="D4">
-        <v>140.4</v>
+        <v>123.55</v>
       </c>
       <c r="E4">
-        <v>140.4</v>
+        <v>247.1</v>
       </c>
       <c r="F4">
-        <v>96.89999999999999</v>
+        <v>87.3</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="H4" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="I4" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -2427,202 +2519,202 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C5">
         <v>1</v>
       </c>
       <c r="D5">
-        <v>139.16</v>
+        <v>122.45</v>
       </c>
       <c r="E5">
-        <v>139.16</v>
+        <v>244.9</v>
       </c>
       <c r="F5">
-        <v>95.89999999999999</v>
+        <v>86.2</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="H5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I5" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D6">
-        <v>126.56</v>
+        <v>128.97</v>
       </c>
       <c r="E6">
-        <v>126.56</v>
+        <v>257.94</v>
       </c>
       <c r="F6">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="G6">
-        <v>0.3</v>
+        <v>1.3</v>
       </c>
       <c r="H6" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:9">
       <c r="A7" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="D7">
-        <v>118.96</v>
+        <v>122.33</v>
       </c>
       <c r="E7">
-        <v>118.96</v>
+        <v>244.66</v>
       </c>
       <c r="F7">
-        <v>57.3</v>
+        <v>69.39999999999999</v>
       </c>
       <c r="G7">
-        <v>0.5</v>
+        <v>2.7</v>
       </c>
       <c r="H7" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="I7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="1" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C8">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D8">
-        <v>120.02</v>
+        <v>113.89</v>
       </c>
       <c r="E8">
-        <v>120.02</v>
+        <v>227.78</v>
       </c>
       <c r="F8">
-        <v>39.8</v>
+        <v>34</v>
       </c>
       <c r="G8">
-        <v>2.1</v>
+        <v>8.9</v>
       </c>
       <c r="H8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I8" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" s="1" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B9" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C9">
         <v>0</v>
       </c>
       <c r="D9">
-        <v>117.86</v>
+        <v>113.63</v>
       </c>
       <c r="E9">
-        <v>117.86</v>
+        <v>227.26</v>
       </c>
       <c r="F9">
-        <v>31.6</v>
+        <v>33.2</v>
       </c>
       <c r="G9">
-        <v>2.4</v>
+        <v>15.5</v>
       </c>
       <c r="H9" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I9" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="10" spans="1:9">
       <c r="A10" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C10">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D10">
-        <v>107</v>
+        <v>102.98</v>
       </c>
       <c r="E10">
-        <v>107</v>
+        <v>205.96</v>
       </c>
       <c r="F10">
-        <v>10.2</v>
+        <v>14.2</v>
       </c>
       <c r="G10">
-        <v>9.1</v>
+        <v>30.7</v>
       </c>
       <c r="H10" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I10" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="11" spans="1:9">
       <c r="A11" s="1" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B11" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C11">
         <v>0</v>
       </c>
       <c r="D11">
-        <v>84.09999999999999</v>
+        <v>107.22</v>
       </c>
       <c r="E11">
-        <v>84.09999999999999</v>
+        <v>214.44</v>
       </c>
       <c r="F11">
-        <v>0.2</v>
+        <v>10.9</v>
       </c>
       <c r="G11">
-        <v>85.59999999999999</v>
+        <v>38.9</v>
       </c>
       <c r="H11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I11" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -2637,19 +2729,19 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="B1" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -2657,19 +2749,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D2">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="E2" t="s">
         <v>11</v>
       </c>
-      <c r="F2">
-        <v>0</v>
+      <c r="F2" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -2677,19 +2769,19 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="D3">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="F3" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -2697,19 +2789,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4">
         <v>5</v>
       </c>
-      <c r="C4" t="s">
-        <v>46</v>
-      </c>
-      <c r="D4">
-        <v>4</v>
-      </c>
       <c r="E4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
+        <v>11</v>
+      </c>
+      <c r="F4" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -2717,19 +2809,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5">
-        <v>0</v>
+        <v>12</v>
+      </c>
+      <c r="F5" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -2737,10 +2829,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C6" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -2748,8 +2840,8 @@
       <c r="E6" t="s">
         <v>11</v>
       </c>
-      <c r="F6">
-        <v>0</v>
+      <c r="F6" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -2757,19 +2849,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D7">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="E7" t="s">
         <v>11</v>
       </c>
-      <c r="F7">
-        <v>0</v>
+      <c r="F7" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -2777,19 +2869,19 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C8" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D8">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="E8" t="s">
-        <v>10</v>
-      </c>
-      <c r="F8">
-        <v>0</v>
+        <v>11</v>
+      </c>
+      <c r="F8" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -2797,19 +2889,19 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D9">
-        <v>-4</v>
+        <v>-6</v>
       </c>
       <c r="E9" t="s">
-        <v>10</v>
-      </c>
-      <c r="F9">
-        <v>0</v>
+        <v>12</v>
+      </c>
+      <c r="F9" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -2817,19 +2909,19 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="C10" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D10">
-        <v>-4</v>
+        <v>-8</v>
       </c>
       <c r="E10" t="s">
-        <v>11</v>
-      </c>
-      <c r="F10">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="F10" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -2837,19 +2929,19 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C11" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D11">
-        <v>-6</v>
+        <v>-11</v>
       </c>
       <c r="E11" t="s">
-        <v>10</v>
-      </c>
-      <c r="F11">
-        <v>0</v>
+        <v>11</v>
+      </c>
+      <c r="F11" t="s">
+        <v>88</v>
       </c>
     </row>
   </sheetData>
@@ -2859,125 +2951,158 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:4">
       <c r="B1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2">
+        <v>4</v>
+      </c>
+      <c r="C2">
+        <v>14</v>
+      </c>
+      <c r="D2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3">
+        <v>-1</v>
+      </c>
+      <c r="C3">
+        <v>7</v>
+      </c>
+      <c r="D3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B2">
+      <c r="B4">
         <v>6</v>
       </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="1" t="s">
+      <c r="C4">
+        <v>5</v>
+      </c>
+      <c r="D4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
+      <c r="B5">
         <v>4</v>
       </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4">
-        <v>4</v>
-      </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" s="1" t="s">
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" s="1" t="s">
-        <v>7</v>
       </c>
       <c r="B6">
         <v>1</v>
       </c>
       <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>-2</v>
+      </c>
+      <c r="D7" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8">
+        <v>-4</v>
+      </c>
+      <c r="C8">
+        <v>-2</v>
+      </c>
+      <c r="D8" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9">
+        <v>-1</v>
+      </c>
+      <c r="C9">
+        <v>-6</v>
+      </c>
+      <c r="D9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B7">
-        <v>-1</v>
-      </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B8">
-        <v>-1</v>
-      </c>
-      <c r="C8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9">
+      <c r="B10">
+        <v>-6</v>
+      </c>
+      <c r="C10">
+        <v>-8</v>
+      </c>
+      <c r="D10" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11">
         <v>-4</v>
       </c>
-      <c r="C9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10">
-        <v>-4</v>
-      </c>
-      <c r="C10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3">
-      <c r="A11" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B11">
-        <v>-6</v>
-      </c>
       <c r="C11">
-        <v>0</v>
+        <v>-11</v>
+      </c>
+      <c r="D11" t="s">
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>